<commit_message>
chore: update react examples
</commit_message>
<xml_diff>
--- a/examples/node/contacts.xlsx
+++ b/examples/node/contacts.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="103">
   <si>
     <t>Id</t>
   </si>
@@ -28,301 +28,298 @@
     <t>Address</t>
   </si>
   <si>
-    <t>Abel Conroy</t>
-  </si>
-  <si>
-    <t>fidget</t>
-  </si>
-  <si>
-    <t>past</t>
-  </si>
-  <si>
-    <t>320 Park Street</t>
-  </si>
-  <si>
-    <t>Opal Strosin</t>
-  </si>
-  <si>
-    <t>indolent</t>
-  </si>
-  <si>
-    <t>robust</t>
-  </si>
-  <si>
-    <t>12469 Marco Manor</t>
-  </si>
-  <si>
-    <t>Luis Murazik</t>
-  </si>
-  <si>
-    <t>nor</t>
-  </si>
-  <si>
-    <t>or</t>
-  </si>
-  <si>
-    <t>253 Hermiston Plains</t>
-  </si>
-  <si>
-    <t>Ramon Davis</t>
-  </si>
-  <si>
-    <t>likable</t>
-  </si>
-  <si>
-    <t>73444 E Pine Street</t>
-  </si>
-  <si>
-    <t>Felix Flatley II</t>
-  </si>
-  <si>
-    <t>militate</t>
-  </si>
-  <si>
-    <t>because</t>
-  </si>
-  <si>
-    <t>643 S 14th Street</t>
-  </si>
-  <si>
-    <t>May Lockman</t>
-  </si>
-  <si>
-    <t>settle</t>
-  </si>
-  <si>
-    <t>gloom</t>
-  </si>
-  <si>
-    <t>360 Breana Views</t>
-  </si>
-  <si>
-    <t>Jaime Greenholt</t>
-  </si>
-  <si>
-    <t>apud</t>
-  </si>
-  <si>
-    <t>extricate</t>
-  </si>
-  <si>
-    <t>87490 Major River</t>
-  </si>
-  <si>
-    <t>Max Koss</t>
-  </si>
-  <si>
-    <t>react</t>
-  </si>
-  <si>
-    <t>gloat</t>
-  </si>
-  <si>
-    <t>517 Terrence Causeway</t>
-  </si>
-  <si>
-    <t>Miss Charlotte Dach</t>
-  </si>
-  <si>
-    <t>where</t>
+    <t>Mariam Greenholt</t>
+  </si>
+  <si>
+    <t>blah</t>
+  </si>
+  <si>
+    <t>sympathetically</t>
+  </si>
+  <si>
+    <t>48366 Jarvis Forest</t>
+  </si>
+  <si>
+    <t>Mrs. Patricia Sipes DVM</t>
+  </si>
+  <si>
+    <t>boiling</t>
+  </si>
+  <si>
+    <t>lively</t>
+  </si>
+  <si>
+    <t>80634 Homenick Cliffs</t>
+  </si>
+  <si>
+    <t>Paul Jenkins</t>
+  </si>
+  <si>
+    <t>weird</t>
+  </si>
+  <si>
+    <t>during</t>
+  </si>
+  <si>
+    <t>6435 Brittany Groves</t>
+  </si>
+  <si>
+    <t>Camila Willms-Emard MD</t>
+  </si>
+  <si>
+    <t>square</t>
+  </si>
+  <si>
+    <t>massage</t>
+  </si>
+  <si>
+    <t>374 Lueilwitz Way</t>
+  </si>
+  <si>
+    <t>Ms. Summer Swift</t>
+  </si>
+  <si>
+    <t>so</t>
+  </si>
+  <si>
+    <t>jot</t>
+  </si>
+  <si>
+    <t>89987 Station Street</t>
+  </si>
+  <si>
+    <t>Marie Hudson</t>
+  </si>
+  <si>
+    <t>lost</t>
+  </si>
+  <si>
+    <t>ravage</t>
+  </si>
+  <si>
+    <t>307 Bartoletti Lake</t>
+  </si>
+  <si>
+    <t>Katie Koelpin III</t>
+  </si>
+  <si>
+    <t>ridge</t>
+  </si>
+  <si>
+    <t>in</t>
+  </si>
+  <si>
+    <t>32521 S College Street</t>
+  </si>
+  <si>
+    <t>Leticia Hodkiewicz</t>
+  </si>
+  <si>
+    <t>serenade</t>
+  </si>
+  <si>
+    <t>structure</t>
+  </si>
+  <si>
+    <t>367 Lincoln Road</t>
+  </si>
+  <si>
+    <t>Hattie Schneider</t>
+  </si>
+  <si>
+    <t>pop</t>
+  </si>
+  <si>
+    <t>dearly</t>
+  </si>
+  <si>
+    <t>4804 Considine Mount</t>
+  </si>
+  <si>
+    <t>Maggie Legros</t>
+  </si>
+  <si>
+    <t>since</t>
+  </si>
+  <si>
+    <t>round</t>
+  </si>
+  <si>
+    <t>789 Quigley Curve</t>
+  </si>
+  <si>
+    <t>Jessica Wehner</t>
+  </si>
+  <si>
+    <t>dead</t>
+  </si>
+  <si>
+    <t>58538 S College Street</t>
+  </si>
+  <si>
+    <t>Lena Ruecker</t>
+  </si>
+  <si>
+    <t>outsource</t>
+  </si>
+  <si>
+    <t>fooey</t>
+  </si>
+  <si>
+    <t>9310 Abbey Road</t>
+  </si>
+  <si>
+    <t>Kian Grant</t>
+  </si>
+  <si>
+    <t>solidly</t>
+  </si>
+  <si>
+    <t>onto</t>
+  </si>
+  <si>
+    <t>741 Gutkowski Courts</t>
+  </si>
+  <si>
+    <t>Bennie Stokes</t>
+  </si>
+  <si>
+    <t>incidentally</t>
+  </si>
+  <si>
+    <t>as</t>
+  </si>
+  <si>
+    <t>8931 West Street</t>
+  </si>
+  <si>
+    <t>Berry Pouros</t>
+  </si>
+  <si>
+    <t>eventually</t>
+  </si>
+  <si>
+    <t>gallery</t>
+  </si>
+  <si>
+    <t>5842 Larch Close</t>
+  </si>
+  <si>
+    <t>Thomas Considine</t>
+  </si>
+  <si>
+    <t>decongestant</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>88826 Wellington Branch</t>
+  </si>
+  <si>
+    <t>Aidan Lindgren</t>
+  </si>
+  <si>
+    <t>willing</t>
+  </si>
+  <si>
+    <t>gadzooks</t>
+  </si>
+  <si>
+    <t>7040 Myrtie Place</t>
+  </si>
+  <si>
+    <t>Sedrick Carroll</t>
+  </si>
+  <si>
+    <t>fuzzy</t>
+  </si>
+  <si>
+    <t>ah</t>
+  </si>
+  <si>
+    <t>424 Mohr Street</t>
+  </si>
+  <si>
+    <t>Johan Howell</t>
+  </si>
+  <si>
+    <t>wholly</t>
+  </si>
+  <si>
+    <t>2710 Grange Close</t>
+  </si>
+  <si>
+    <t>Sonja Larson</t>
+  </si>
+  <si>
+    <t>ick</t>
+  </si>
+  <si>
+    <t>prioritize</t>
+  </si>
+  <si>
+    <t>37428 Ruecker Plains</t>
+  </si>
+  <si>
+    <t>Mr. Hugo Schaden</t>
+  </si>
+  <si>
+    <t>hope</t>
+  </si>
+  <si>
+    <t>ultimately</t>
+  </si>
+  <si>
+    <t>96840 Carmen Station</t>
+  </si>
+  <si>
+    <t>Jerome Kovacek</t>
+  </si>
+  <si>
+    <t>without</t>
+  </si>
+  <si>
+    <t>pronoun</t>
+  </si>
+  <si>
+    <t>73708 Bartell Corners</t>
+  </si>
+  <si>
+    <t>Dr. Hans Quitzon</t>
+  </si>
+  <si>
+    <t>fashion</t>
+  </si>
+  <si>
+    <t>unto</t>
+  </si>
+  <si>
+    <t>1377 Kozey Estate</t>
+  </si>
+  <si>
+    <t>Arlene Gibson II</t>
   </si>
   <si>
     <t>but</t>
   </si>
   <si>
-    <t>22874 Halvorson River</t>
-  </si>
-  <si>
-    <t>Rolando Bernhard</t>
-  </si>
-  <si>
-    <t>yowza</t>
-  </si>
-  <si>
-    <t>step-mother</t>
-  </si>
-  <si>
-    <t>43891 Orn Throughway</t>
-  </si>
-  <si>
-    <t>Earl Price</t>
-  </si>
-  <si>
-    <t>supposing</t>
-  </si>
-  <si>
-    <t>nutritious</t>
-  </si>
-  <si>
-    <t>454 Rutherford Rest</t>
-  </si>
-  <si>
-    <t>Simon Hegmann-Langworth</t>
-  </si>
-  <si>
-    <t>acknowledge</t>
-  </si>
-  <si>
-    <t>next</t>
-  </si>
-  <si>
-    <t>4281 Heaney Terrace</t>
-  </si>
-  <si>
-    <t>Tyler Tromp III</t>
-  </si>
-  <si>
-    <t>dishearten</t>
-  </si>
-  <si>
-    <t>brandish</t>
-  </si>
-  <si>
-    <t>748 Roman Way</t>
-  </si>
-  <si>
-    <t>Casey Satterfield</t>
-  </si>
-  <si>
-    <t>loyally</t>
-  </si>
-  <si>
-    <t>likewise</t>
-  </si>
-  <si>
-    <t>4899 N Court Street</t>
-  </si>
-  <si>
-    <t>Dave Mann</t>
-  </si>
-  <si>
-    <t>thoroughly</t>
-  </si>
-  <si>
-    <t>enormously</t>
-  </si>
-  <si>
-    <t>8045 Miller Vista</t>
-  </si>
-  <si>
-    <t>Timothy Hudson</t>
-  </si>
-  <si>
-    <t>until</t>
-  </si>
-  <si>
-    <t>only</t>
-  </si>
-  <si>
-    <t>388 Johnson Street</t>
-  </si>
-  <si>
-    <t>Bennie Mertz</t>
-  </si>
-  <si>
-    <t>typeface</t>
-  </si>
-  <si>
-    <t>curse</t>
-  </si>
-  <si>
-    <t>285 Edyth Avenue</t>
-  </si>
-  <si>
-    <t>Irma Bogisich</t>
-  </si>
-  <si>
-    <t>the</t>
-  </si>
-  <si>
-    <t>jellyfish</t>
-  </si>
-  <si>
-    <t>3300 Hammes Harbor</t>
-  </si>
-  <si>
-    <t>Ollie Nikolaus</t>
-  </si>
-  <si>
-    <t>although</t>
-  </si>
-  <si>
-    <t>too</t>
-  </si>
-  <si>
-    <t>93795 N 5th Street</t>
-  </si>
-  <si>
-    <t>Karla Boyer</t>
-  </si>
-  <si>
-    <t>adventurously</t>
-  </si>
-  <si>
-    <t>ultimately</t>
-  </si>
-  <si>
-    <t>11780 Nader Cove</t>
-  </si>
-  <si>
-    <t>Roderick Dietrich</t>
-  </si>
-  <si>
-    <t>unimpressively</t>
-  </si>
-  <si>
-    <t>whose</t>
-  </si>
-  <si>
-    <t>9022 Hazel Grove</t>
-  </si>
-  <si>
-    <t>Jo Berge</t>
-  </si>
-  <si>
-    <t>exotic</t>
-  </si>
-  <si>
-    <t>inasmuch</t>
-  </si>
-  <si>
-    <t>10146 Runte Trace</t>
-  </si>
-  <si>
-    <t>Brooke Tremblay</t>
-  </si>
-  <si>
-    <t>hoof</t>
-  </si>
-  <si>
-    <t>replacement</t>
-  </si>
-  <si>
-    <t>7210 Hilpert Lane</t>
-  </si>
-  <si>
-    <t>Sandy Hickle</t>
-  </si>
-  <si>
-    <t>aside</t>
-  </si>
-  <si>
-    <t>foolhardy</t>
-  </si>
-  <si>
-    <t>90379 Nienow Valleys</t>
-  </si>
-  <si>
-    <t>Jerald Cummerata</t>
-  </si>
-  <si>
-    <t>offensively</t>
-  </si>
-  <si>
-    <t>during</t>
-  </si>
-  <si>
-    <t>37298 Myrna Villages</t>
+    <t>till</t>
+  </si>
+  <si>
+    <t>27822 Main Street E</t>
+  </si>
+  <si>
+    <t>Osborne Stoltenberg-Pfeffer</t>
+  </si>
+  <si>
+    <t>yearningly</t>
+  </si>
+  <si>
+    <t>if</t>
+  </si>
+  <si>
+    <t>9025 Kacie Rue</t>
   </si>
 </sst>
 </file>
@@ -712,10 +709,10 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -797,10 +794,10 @@
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -808,16 +805,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -825,16 +822,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -842,16 +839,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -859,16 +856,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -876,16 +873,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -893,16 +890,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -910,13 +907,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="E12" t="s">
         <v>47</v>
@@ -1052,10 +1049,10 @@
         <v>77</v>
       </c>
       <c r="D20" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" t="s">
         <v>78</v>
-      </c>
-      <c r="E20" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1063,16 +1060,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s">
         <v>80</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>81</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>82</v>
-      </c>
-      <c r="E21" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1080,16 +1077,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" t="s">
         <v>84</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>85</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>86</v>
-      </c>
-      <c r="E22" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1097,16 +1094,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" t="s">
         <v>88</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>89</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>90</v>
-      </c>
-      <c r="E23" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1114,16 +1111,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" t="s">
         <v>92</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>93</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>94</v>
-      </c>
-      <c r="E24" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1131,16 +1128,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" t="s">
         <v>96</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>97</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>98</v>
-      </c>
-      <c r="E25" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1148,16 +1145,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" t="s">
         <v>100</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>101</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>102</v>
-      </c>
-      <c r="E26" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>